<commit_message>
correcion de errores y pulido de la vista SelecList
</commit_message>
<xml_diff>
--- a/LISTAS/ma/ROLDANAS DISMAY.xlsx
+++ b/LISTAS/ma/ROLDANAS DISMAY.xlsx
@@ -790,14 +790,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="14" t="n">
-        <v>45163.60914307342</v>
+        <v>45211</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="22.5" customHeight="1" s="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -843,21 +839,6 @@
       </c>
       <c r="E11" s="9" t="n"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
     <row r="27" ht="18" customHeight="1" s="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
@@ -889,7 +870,7 @@
       </c>
       <c r="C28" s="23" t="n"/>
       <c r="D28" s="24" t="n">
-        <v>93.33</v>
+        <v>160</v>
       </c>
       <c r="E28" s="25" t="n"/>
       <c r="F28" s="26" t="n"/>
@@ -948,18 +929,6 @@
       <c r="E31" s="25" t="n"/>
       <c r="F31" s="26" t="n"/>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
     <row r="44" ht="15" customHeight="1" s="1">
       <c r="A44" s="18" t="inlineStr">
         <is>
@@ -977,15 +946,15 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="B27:C27"/>
+    <mergeCell ref="A10:D10"/>
     <mergeCell ref="A44:D44"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="A11:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
haciendo la vista descargas para descargar las listas
</commit_message>
<xml_diff>
--- a/LISTAS/ma/ROLDANAS DISMAY.xlsx
+++ b/LISTAS/ma/ROLDANAS DISMAY.xlsx
@@ -790,7 +790,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="14" t="n">
-        <v>45214</v>
+        <v>45216</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
@@ -870,7 +870,7 @@
       </c>
       <c r="C28" s="23" t="n"/>
       <c r="D28" s="24" t="n">
-        <v>193.6</v>
+        <v>130</v>
       </c>
       <c r="E28" s="25" t="n"/>
       <c r="F28" s="26" t="n"/>
@@ -888,7 +888,7 @@
       </c>
       <c r="C29" s="23" t="n"/>
       <c r="D29" s="24" t="n">
-        <v>121.4</v>
+        <v>140</v>
       </c>
       <c r="E29" s="25" t="n"/>
       <c r="F29" s="26" t="n"/>
@@ -924,7 +924,7 @@
       </c>
       <c r="C31" s="23" t="n"/>
       <c r="D31" s="24" t="n">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="E31" s="25" t="n"/>
       <c r="F31" s="26" t="n"/>

</xml_diff>